<commit_message>
Corrida | SFE-IND2 | 2026-04-28 10:19:39.182683
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND2_out.xlsx
+++ b/indicadores/SFE-IND2_out.xlsx
@@ -107,7 +107,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">06/04/2026</t>
+    <t xml:space="preserve">28/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1652,7 +1652,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.578134592638628</v>
+        <v>0.575184585889915</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1710,7 +1710,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.299581339926856</v>
+        <v>0.297333675051944</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1780,7 +1780,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.006597198725895</v>
+        <v>0.00600503958007607</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1810,7 +1810,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0925057822730915</v>
+        <v>0.0880260006205179</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -16451,7 +16451,7 @@
         <v>349</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0575985435945254</v>
+        <v>-0.0607677912331837</v>
       </c>
     </row>
     <row r="6">
@@ -16459,7 +16459,7 @@
         <v>350</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0589057188055645</v>
+        <v>-0.0615418663985872</v>
       </c>
     </row>
     <row r="7">
@@ -16467,7 +16467,7 @@
         <v>351</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.0394281150858759</v>
+        <v>-0.037319630254014</v>
       </c>
     </row>
     <row r="8">
@@ -16475,7 +16475,7 @@
         <v>352</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0971103803657381</v>
+        <v>0.102541598489879</v>
       </c>
     </row>
     <row r="9">
@@ -16483,7 +16483,7 @@
         <v>353</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.256343988568903</v>
+        <v>0.259590613012012</v>
       </c>
     </row>
     <row r="10">
@@ -16491,7 +16491,7 @@
         <v>354</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.359506630823727</v>
+        <v>0.360523693049197</v>
       </c>
     </row>
     <row r="11">
@@ -16499,7 +16499,7 @@
         <v>355</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.447893041128027</v>
+        <v>0.447674377701817</v>
       </c>
     </row>
     <row r="12">
@@ -16507,7 +16507,7 @@
         <v>356</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.537096055882144</v>
+        <v>0.53424417219226</v>
       </c>
     </row>
     <row r="13">
@@ -16515,7 +16515,7 @@
         <v>357</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.578134592638628</v>
+        <v>0.575184585889915</v>
       </c>
     </row>
     <row r="14">
@@ -16523,7 +16523,7 @@
         <v>358</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.547340241464901</v>
+        <v>0.54528311458539</v>
       </c>
     </row>
     <row r="15">
@@ -16531,7 +16531,7 @@
         <v>359</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.440808824808234</v>
+        <v>0.437278429352245</v>
       </c>
     </row>
     <row r="16">
@@ -16539,7 +16539,7 @@
         <v>360</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.325486902117541</v>
+        <v>0.323128789780989</v>
       </c>
     </row>
     <row r="17">
@@ -16547,7 +16547,7 @@
         <v>361</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.248836714817055</v>
+        <v>0.250201151153955</v>
       </c>
     </row>
     <row r="18">
@@ -16555,7 +16555,7 @@
         <v>362</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.171128108361567</v>
+        <v>0.173736908761512</v>
       </c>
     </row>
     <row r="19">
@@ -16563,7 +16563,7 @@
         <v>363</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0798968271014397</v>
+        <v>0.0811511037810239</v>
       </c>
     </row>
     <row r="20">
@@ -16571,7 +16571,7 @@
         <v>364</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0232974270256893</v>
+        <v>-0.0230355873808223</v>
       </c>
     </row>
     <row r="21">
@@ -16579,7 +16579,7 @@
         <v>365</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.109017558808138</v>
+        <v>-0.109548190698682</v>
       </c>
     </row>
     <row r="22">
@@ -16587,7 +16587,7 @@
         <v>366</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.187347518512776</v>
+        <v>-0.189915719907711</v>
       </c>
     </row>
     <row r="23">
@@ -16595,7 +16595,7 @@
         <v>367</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.254238635214983</v>
+        <v>-0.257135453021291</v>
       </c>
     </row>
     <row r="24">
@@ -16623,4 +16623,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D08DC829-AFE2-4E6F-985E-EC351BF6C5F3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C3FB808-8B2F-4D75-A777-14844248271D}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3780BD2-ACE9-4978-A998-97A3E15ECE99}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-IND2 | 2026-05-27 10:52:06.31075
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND2_out.xlsx
+++ b/indicadores/SFE-IND2_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">04/05/2026</t>
+    <t xml:space="preserve">27/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1652,7 +1652,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.574119309730337</v>
+        <v>0.577565823104832</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1710,7 +1710,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.310817742940142</v>
+        <v>0.306510812462396</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1780,7 +1780,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00579899291568458</v>
+        <v>0.00321984009552446</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1810,7 +1810,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.035375828162574</v>
+        <v>0.0399380072782171</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -16487,7 +16487,7 @@
         <v>349</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0623224905521082</v>
+        <v>-0.0755585648088104</v>
       </c>
     </row>
     <row r="6">
@@ -16495,7 +16495,7 @@
         <v>350</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0507027180533029</v>
+        <v>-0.054594241564003</v>
       </c>
     </row>
     <row r="7">
@@ -16503,7 +16503,7 @@
         <v>351</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.0227757966477548</v>
+        <v>-0.0223638318231945</v>
       </c>
     </row>
     <row r="8">
@@ -16511,7 +16511,7 @@
         <v>352</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0929145208612996</v>
+        <v>0.091300295677357</v>
       </c>
     </row>
     <row r="9">
@@ -16519,7 +16519,7 @@
         <v>353</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.221307741740602</v>
+        <v>0.222023132808281</v>
       </c>
     </row>
     <row r="10">
@@ -16527,7 +16527,7 @@
         <v>354</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.33389119720106</v>
+        <v>0.333962224312283</v>
       </c>
     </row>
     <row r="11">
@@ -16535,7 +16535,7 @@
         <v>355</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.453009691091671</v>
+        <v>0.455096003148631</v>
       </c>
     </row>
     <row r="12">
@@ -16543,7 +16543,7 @@
         <v>356</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.540460200012925</v>
+        <v>0.548192347487697</v>
       </c>
     </row>
     <row r="13">
@@ -16551,7 +16551,7 @@
         <v>357</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.574119309730337</v>
+        <v>0.577565823104832</v>
       </c>
     </row>
     <row r="14">
@@ -16559,7 +16559,7 @@
         <v>358</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.557510307474347</v>
+        <v>0.553634186500794</v>
       </c>
     </row>
     <row r="15">
@@ -16567,7 +16567,7 @@
         <v>359</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.460032358778911</v>
+        <v>0.455230877757664</v>
       </c>
     </row>
     <row r="16">
@@ -16575,7 +16575,7 @@
         <v>360</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.33750268367008</v>
+        <v>0.332395110450836</v>
       </c>
     </row>
     <row r="17">
@@ -16583,7 +16583,7 @@
         <v>361</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.251869852794792</v>
+        <v>0.244154625373639</v>
       </c>
     </row>
     <row r="18">
@@ -16591,7 +16591,7 @@
         <v>362</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.165100993689284</v>
+        <v>0.166983650595509</v>
       </c>
     </row>
     <row r="19">
@@ -16599,7 +16599,7 @@
         <v>363</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0814999000220871</v>
+        <v>0.0937076123963772</v>
       </c>
     </row>
     <row r="20">
@@ -16607,7 +16607,7 @@
         <v>364</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.00441991863699993</v>
+        <v>-0.000463363421597884</v>
       </c>
     </row>
     <row r="21">
@@ -16615,7 +16615,7 @@
         <v>365</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0762041853858826</v>
+        <v>-0.08161301104008</v>
       </c>
     </row>
     <row r="22">
@@ -16623,7 +16623,7 @@
         <v>366</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.15137825191612</v>
+        <v>-0.149626862475376</v>
       </c>
     </row>
     <row r="23">
@@ -16631,7 +16631,7 @@
         <v>367</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.238203473184658</v>
+        <v>-0.232113353717459</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-IND2 | 2026-06-17 12:04:30.174585
</commit_message>
<xml_diff>
--- a/indicadores/SFE-IND2_out.xlsx
+++ b/indicadores/SFE-IND2_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="370">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice de producción industrial de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Índice de producción industrial</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">01/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1620,9 +1626,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1633,7 +1643,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1647,7 +1657,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1663,7 +1673,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1691,7 +1701,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1705,7 +1715,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1733,7 +1743,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1747,7 +1757,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1761,7 +1771,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1775,7 +1785,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1791,7 +1801,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1805,7 +1815,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1953,10 +1963,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1969,10 +1979,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1996,66 +2006,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>98.2277820753913</v>
@@ -2108,7 +2118,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>90.123779283495</v>
@@ -2165,7 +2175,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>82.428656294783</v>
@@ -2222,7 +2232,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>111.627937833908</v>
@@ -2279,7 +2289,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>116.182979695205</v>
@@ -2336,7 +2346,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>92.8296434744574</v>
@@ -2393,7 +2403,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>112.507498616931</v>
@@ -2450,7 +2460,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>105.233652349113</v>
@@ -2507,7 +2517,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>114.099526476341</v>
@@ -2564,7 +2574,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>100.127208367592</v>
@@ -2621,7 +2631,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>90.2176770524802</v>
@@ -2678,7 +2688,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>86.3936584803029</v>
@@ -2735,7 +2745,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>75.2420443340881</v>
@@ -2794,7 +2804,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>71.1027619225755</v>
@@ -2853,7 +2863,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>76.7339809122391</v>
@@ -2912,7 +2922,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>89.5758734148106</v>
@@ -2971,7 +2981,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>86.623484420718</v>
@@ -3030,7 +3040,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>96.1337952744985</v>
@@ -3089,7 +3099,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>88.4443855037097</v>
@@ -3148,7 +3158,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>88.4778988206624</v>
@@ -3207,7 +3217,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>91.868393504618</v>
@@ -3266,7 +3276,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>92.0999923354386</v>
@@ -3325,7 +3335,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>85.942752427295</v>
@@ -3384,7 +3394,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>88.167165912867</v>
@@ -3443,7 +3453,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>81.3588524071837</v>
@@ -3502,7 +3512,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>74.0804856727769</v>
@@ -3561,7 +3571,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>82.3241167299284</v>
@@ -3620,7 +3630,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>109.591836868308</v>
@@ -3679,7 +3689,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>98.1673031365672</v>
@@ -3738,7 +3748,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>99.8546670433968</v>
@@ -3797,7 +3807,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>101.149951000052</v>
@@ -3856,7 +3866,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>103.441613103028</v>
@@ -3915,7 +3925,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>109.501685323641</v>
@@ -3974,7 +3984,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>102.953595316765</v>
@@ -4033,7 +4043,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>107.769849806298</v>
@@ -4092,7 +4102,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>100.479436850124</v>
@@ -4151,7 +4161,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>93.2334112344005</v>
@@ -4210,7 +4220,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>84.1989088526031</v>
@@ -4269,7 +4279,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>94.1349889497777</v>
@@ -4328,7 +4338,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>103.96735971976</v>
@@ -4387,7 +4397,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>114.46764998704</v>
@@ -4446,7 +4456,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>103.664529628861</v>
@@ -4505,7 +4515,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>117.452679644761</v>
@@ -4564,7 +4574,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>105.628116040907</v>
@@ -4623,7 +4633,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>111.679766878388</v>
@@ -4682,7 +4692,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>98.2361924848471</v>
@@ -4741,7 +4751,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>106.199003515125</v>
@@ -4800,7 +4810,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>98.7085995450217</v>
@@ -4859,7 +4869,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>79.2219113231338</v>
@@ -4918,7 +4928,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>87.0654200388252</v>
@@ -4977,7 +4987,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>95.5448890311325</v>
@@ -5036,7 +5046,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>95.8128459233493</v>
@@ -5095,7 +5105,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>102.120778062452</v>
@@ -5154,7 +5164,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>101.033772360959</v>
@@ -5213,7 +5223,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>96.9275634528426</v>
@@ -5272,7 +5282,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>109.017131885614</v>
@@ -5331,7 +5341,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>96.5741957690519</v>
@@ -5390,7 +5400,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>97.9166368395107</v>
@@ -5449,7 +5459,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>96.0480455009746</v>
@@ -5508,7 +5518,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>100.963397880312</v>
@@ -5567,7 +5577,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>76.2589011982098</v>
@@ -5626,7 +5636,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>77.1712232007344</v>
@@ -5685,7 +5695,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>92.325227398488</v>
@@ -5744,7 +5754,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>95.6959545092515</v>
@@ -5803,7 +5813,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>106.889583012614</v>
@@ -5862,7 +5872,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>117.561465424953</v>
@@ -5921,7 +5931,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>108.363912262066</v>
@@ -5980,7 +5990,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>102.648427567053</v>
@@ -6039,7 +6049,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>104.753488551763</v>
@@ -6098,7 +6108,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>107.213136951118</v>
@@ -6157,7 +6167,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>100.264302693548</v>
@@ -6216,7 +6226,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>119.136522692011</v>
@@ -6275,7 +6285,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>83.305576338085</v>
@@ -6334,7 +6344,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>81.4141232556816</v>
@@ -6393,7 +6403,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>90.7117392003981</v>
@@ -6452,7 +6462,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>101.194171866087</v>
@@ -6511,7 +6521,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>107.132824829095</v>
@@ -6570,7 +6580,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>104.060398589074</v>
@@ -6629,7 +6639,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>101.468423727314</v>
@@ -6688,7 +6698,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>98.1622780124311</v>
@@ -6747,7 +6757,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>108.277639100706</v>
@@ -6806,7 +6816,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>104.304408011137</v>
@@ -6865,7 +6875,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>102.809615849083</v>
@@ -6924,7 +6934,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>97.7399148856869</v>
@@ -6983,7 +6993,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>76.1404042238856</v>
@@ -7042,7 +7052,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>78.675207001216</v>
@@ -7101,7 +7111,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>88.6484827691763</v>
@@ -7160,7 +7170,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>104.216712414203</v>
@@ -7219,7 +7229,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>94.0872748104741</v>
@@ -7278,7 +7288,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>114.834193862872</v>
@@ -7337,7 +7347,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>106.341390777791</v>
@@ -7396,7 +7406,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>99.6253435426621</v>
@@ -7455,7 +7465,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>108.674528773825</v>
@@ -7514,7 +7524,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>108.673869910755</v>
@@ -7573,7 +7583,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>102.784515450776</v>
@@ -7632,7 +7642,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>103.260800024495</v>
@@ -7691,7 +7701,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>83.4036739319931</v>
@@ -7750,7 +7760,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>85.2063851122631</v>
@@ -7809,7 +7819,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>98.8143744975921</v>
@@ -7868,7 +7878,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>91.9809773606431</v>
@@ -7927,7 +7937,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>96.0876637221686</v>
@@ -7986,7 +7996,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>97.4106325267393</v>
@@ -8045,7 +8055,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>97.7380351670361</v>
@@ -8104,7 +8114,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>106.278013521967</v>
@@ -8163,7 +8173,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>108.080991851257</v>
@@ -8222,7 +8232,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>99.5889833487838</v>
@@ -8281,7 +8291,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>107.114833051681</v>
@@ -8340,7 +8350,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>105.086673671947</v>
@@ -8399,7 +8409,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>85.8794962678109</v>
@@ -8458,7 +8468,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>86.2057648521377</v>
@@ -8517,7 +8527,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>104.385933037628</v>
@@ -8576,7 +8586,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>102.306726109055</v>
@@ -8635,7 +8645,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>115.604451222519</v>
@@ -8694,7 +8704,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>105.187122405492</v>
@@ -8753,7 +8763,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>106.97399549071</v>
@@ -8812,7 +8822,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>107.956509639225</v>
@@ -8871,7 +8881,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>109.730127224526</v>
@@ -8930,7 +8940,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>112.245781254405</v>
@@ -8989,7 +8999,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>105.853350553335</v>
@@ -9048,7 +9058,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>103.621303036554</v>
@@ -9107,7 +9117,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>93.4016978687685</v>
@@ -9166,7 +9176,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>91.0640005124949</v>
@@ -9225,7 +9235,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>105.863023169303</v>
@@ -9284,7 +9294,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>100.305055375439</v>
@@ -9343,7 +9353,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>105.581616899387</v>
@@ -9402,7 +9412,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>101.857869730298</v>
@@ -9461,7 +9471,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>102.514881598536</v>
@@ -9520,7 +9530,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>102.933423076146</v>
@@ -9579,7 +9589,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>94.5595719534699</v>
@@ -9638,7 +9648,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>97.5507884255321</v>
@@ -9697,7 +9707,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>88.0688615817144</v>
@@ -9756,7 +9766,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>86.3318434069674</v>
@@ -9815,7 +9825,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>79.2748478627445</v>
@@ -9874,7 +9884,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>78.9956094235717</v>
@@ -9933,7 +9943,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>87.9297773214196</v>
@@ -9992,7 +10002,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>92.4606278057285</v>
@@ -10051,7 +10061,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>99.7623903661728</v>
@@ -10110,7 +10120,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>94.0334251887938</v>
@@ -10169,7 +10179,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>102.264455586205</v>
@@ -10228,7 +10238,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>102.110150191835</v>
@@ -10287,7 +10297,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>95.5257332957513</v>
@@ -10346,7 +10356,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>104.476421904702</v>
@@ -10405,7 +10415,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>90.3997238113681</v>
@@ -10464,7 +10474,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>87.9928276913698</v>
@@ -10523,7 +10533,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>74.1376033457939</v>
@@ -10582,7 +10592,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>73.8459708460078</v>
@@ -10641,7 +10651,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>69.4740324008248</v>
@@ -10700,7 +10710,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>70.3846395992028</v>
@@ -10759,7 +10769,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>86.4944582871762</v>
@@ -10818,7 +10828,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>93.4597127241302</v>
@@ -10877,7 +10887,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>90.9782841159934</v>
@@ -10936,7 +10946,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>93.2916455610629</v>
@@ -10995,7 +11005,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>97.2283920277679</v>
@@ -11054,7 +11064,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>98.3720068171732</v>
@@ -11113,7 +11123,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>89.5808943898706</v>
@@ -11172,7 +11182,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>76.8370587951443</v>
@@ -11231,7 +11241,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>84.3195202228677</v>
@@ -11290,7 +11300,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>82.3995814037724</v>
@@ -11349,7 +11359,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>100.342964118279</v>
@@ -11408,7 +11418,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>101.650081288574</v>
@@ -11467,7 +11477,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>96.1317058444843</v>
@@ -11526,7 +11536,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>104.258186087537</v>
@@ -11585,7 +11595,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>105.37249827402</v>
@@ -11644,7 +11654,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>105.699421764708</v>
@@ -11703,7 +11713,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>107.152228440203</v>
@@ -11762,7 +11772,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>105.866773550425</v>
@@ -11821,7 +11831,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>102.39255867579</v>
@@ -11880,7 +11890,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>99.3212747316944</v>
@@ -11939,7 +11949,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>79.8039720303685</v>
@@ -11998,7 +12008,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>90.5888855570312</v>
@@ -12057,7 +12067,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>103.506586602343</v>
@@ -12116,7 +12126,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>107.263449154075</v>
@@ -12175,7 +12185,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>110.359523822292</v>
@@ -12234,7 +12244,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>119.830083570032</v>
@@ -12293,7 +12303,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>108.822009555436</v>
@@ -12352,7 +12362,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>116.506627857385</v>
@@ -12411,7 +12421,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>108.478914649402</v>
@@ -12470,7 +12480,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>107.812864930698</v>
@@ -12529,7 +12539,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>107.086804637541</v>
@@ -12588,7 +12598,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>99.5186317748409</v>
@@ -12647,7 +12657,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>83.9732052225982</v>
@@ -12706,7 +12716,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>82.4443266854149</v>
@@ -12765,7 +12775,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>98.4157013506302</v>
@@ -12824,7 +12834,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>98.6471646185455</v>
@@ -12883,7 +12893,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>107.889092405321</v>
@@ -12942,7 +12952,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>101.585463966791</v>
@@ -13001,7 +13011,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>98.1031749942026</v>
@@ -13060,7 +13070,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>100.892294247782</v>
@@ -13119,7 +13129,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>97.9675659577667</v>
@@ -13178,7 +13188,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>92.4657629020759</v>
@@ -13237,7 +13247,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>81.3677441530628</v>
@@ -13296,7 +13306,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>80.7784045667268</v>
@@ -13355,7 +13365,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>83.0650405476002</v>
@@ -13414,7 +13424,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>77.6793053627653</v>
@@ -13473,7 +13483,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>84.5795910719569</v>
@@ -13532,7 +13542,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>93.8512612030798</v>
@@ -13591,7 +13601,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>97.6482905005603</v>
@@ -13650,7 +13660,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>90.7660322988151</v>
@@ -13709,7 +13719,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>102.198764539754</v>
@@ -13768,7 +13778,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>115.131160743312</v>
@@ -13827,7 +13837,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>114.516784351189</v>
@@ -13886,7 +13896,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>101.450032291191</v>
@@ -13945,7 +13955,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>110.874813986052</v>
@@ -14004,7 +14014,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>102.900800270937</v>
@@ -14063,7 +14073,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>95.4710051744574</v>
@@ -14122,7 +14132,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>88.26319525734</v>
@@ -14181,7 +14191,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>96.6682515198397</v>
@@ -14240,7 +14250,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>104.293125699306</v>
@@ -14299,7 +14309,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>107.213756173358</v>
@@ -14358,7 +14368,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>100.896838326861</v>
@@ -14417,7 +14427,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>118.863931095332</v>
@@ -14476,7 +14486,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>109.397582612121</v>
@@ -14535,7 +14545,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>112.920142044852</v>
@@ -14594,7 +14604,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>111.43078023271</v>
@@ -14653,7 +14663,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>101.982185807202</v>
@@ -14712,7 +14722,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>98.962803967689</v>
@@ -14771,7 +14781,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>98.1963042134765</v>
@@ -14830,7 +14840,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>84.5122177839759</v>
@@ -14889,7 +14899,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>93.776741491578</v>
@@ -14948,7 +14958,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2"/>
       <c r="C221" s="3" t="n">
@@ -14981,7 +14991,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2"/>
       <c r="C222" s="3" t="n">
@@ -15014,7 +15024,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2"/>
       <c r="C223" s="3" t="n">
@@ -15047,7 +15057,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2"/>
       <c r="C224" s="3" t="n">
@@ -15080,7 +15090,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2"/>
       <c r="C225" s="3" t="n">
@@ -15113,7 +15123,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2"/>
       <c r="C226" s="3" t="n">
@@ -15146,7 +15156,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="3" t="n">
@@ -15179,7 +15189,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2"/>
       <c r="C228" s="3" t="n">
@@ -15212,7 +15222,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2"/>
       <c r="C229" s="3" t="n">
@@ -15245,7 +15255,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2"/>
       <c r="C230" s="3" t="n">
@@ -15278,7 +15288,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2"/>
       <c r="C231" s="3" t="n">
@@ -15311,7 +15321,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2"/>
       <c r="C232" s="3" t="n">
@@ -15344,7 +15354,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2"/>
       <c r="C233" s="3"/>
@@ -15367,7 +15377,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2"/>
       <c r="C234" s="3"/>
@@ -15390,7 +15400,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2"/>
       <c r="C235" s="3"/>
@@ -15413,7 +15423,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2"/>
       <c r="C236" s="3"/>
@@ -15436,7 +15446,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2"/>
       <c r="C237" s="3"/>
@@ -15459,7 +15469,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2"/>
       <c r="C238" s="3"/>
@@ -15482,7 +15492,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="3"/>
@@ -15505,7 +15515,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2"/>
       <c r="C240" s="3"/>
@@ -15528,7 +15538,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2"/>
       <c r="C241" s="3"/>
@@ -15551,7 +15561,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2"/>
       <c r="C242" s="3"/>
@@ -15574,7 +15584,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2"/>
       <c r="C243" s="3"/>
@@ -15597,7 +15607,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2"/>
       <c r="C244" s="3"/>
@@ -15620,7 +15630,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2"/>
       <c r="C245" s="3"/>
@@ -15643,7 +15653,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2"/>
       <c r="C246" s="3"/>
@@ -15666,7 +15676,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2"/>
       <c r="C247" s="3"/>
@@ -15689,7 +15699,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2"/>
       <c r="C248" s="3"/>
@@ -15712,7 +15722,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2"/>
       <c r="C249" s="3"/>
@@ -15735,7 +15745,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2"/>
       <c r="C250" s="3"/>
@@ -15758,7 +15768,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2"/>
       <c r="C251" s="3"/>
@@ -15781,7 +15791,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2"/>
       <c r="C252" s="3"/>
@@ -15804,7 +15814,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2"/>
       <c r="C253" s="3"/>
@@ -15827,7 +15837,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2"/>
       <c r="C254" s="3"/>
@@ -15850,7 +15860,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2"/>
       <c r="C255" s="3"/>
@@ -15873,7 +15883,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2"/>
       <c r="C256" s="3"/>
@@ -15896,7 +15906,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2"/>
       <c r="C257" s="3"/>
@@ -15919,7 +15929,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2"/>
       <c r="C258" s="3"/>
@@ -15942,7 +15952,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2"/>
       <c r="C259" s="3"/>
@@ -15965,7 +15975,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2"/>
       <c r="C260" s="3"/>
@@ -15988,7 +15998,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2"/>
       <c r="C261" s="3"/>
@@ -16011,7 +16021,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2"/>
       <c r="C262" s="3"/>
@@ -16034,7 +16044,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2"/>
       <c r="C263" s="3"/>
@@ -16057,7 +16067,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2"/>
       <c r="C264" s="3"/>
@@ -16080,7 +16090,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2"/>
       <c r="C265" s="3"/>
@@ -16103,7 +16113,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2"/>
       <c r="C266" s="3"/>
@@ -16126,7 +16136,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2"/>
       <c r="C267" s="3"/>
@@ -16149,7 +16159,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2"/>
       <c r="C268" s="3"/>
@@ -16172,7 +16182,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2"/>
       <c r="C269" s="3"/>
@@ -16195,7 +16205,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2"/>
       <c r="C270" s="3"/>
@@ -16218,7 +16228,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2"/>
       <c r="C271" s="3"/>
@@ -16241,7 +16251,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2"/>
       <c r="C272" s="3"/>
@@ -16264,7 +16274,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2"/>
       <c r="C273" s="3"/>
@@ -16287,7 +16297,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2"/>
       <c r="C274" s="3"/>
@@ -16310,7 +16320,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2"/>
       <c r="C275" s="3"/>
@@ -16333,7 +16343,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2"/>
       <c r="C276" s="3"/>
@@ -16356,7 +16366,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2"/>
       <c r="C277" s="3"/>
@@ -16390,97 +16400,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -16504,7 +16514,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -16514,13 +16524,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.110215225653635</v>
@@ -16528,7 +16538,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.0930784896756451</v>
@@ -16536,7 +16546,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0318817828627175</v>
@@ -16544,7 +16554,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.0999922944227211</v>
@@ -16552,7 +16562,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.241267056357498</v>
@@ -16560,7 +16570,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.353585666256505</v>
@@ -16568,7 +16578,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.461575910258249</v>
@@ -16576,7 +16586,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.541732422802072</v>
@@ -16584,7 +16594,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.564945813667587</v>
@@ -16592,7 +16602,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.547173109856526</v>
@@ -16600,7 +16610,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.457058968483558</v>
@@ -16608,7 +16618,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.334029082153896</v>
@@ -16616,7 +16626,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.252726229944709</v>
@@ -16624,7 +16634,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.173238669412411</v>
@@ -16632,7 +16642,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.0590975942314088</v>
@@ -16640,7 +16650,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.0817509285578485</v>
@@ -16648,7 +16658,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.17915921840114</v>
@@ -16656,7 +16666,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.226521584465485</v>
@@ -16664,7 +16674,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.279261949792279</v>

</xml_diff>